<commit_message>
Add missing functionality, tests and clean-up files.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_convertiblebonds.xlsx
+++ b/tests/workbooktests/workbooks/test_convertiblebonds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32841E5A-7123-44E6-86B9-437BE0D70700}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F7B273-20F1-49A9-A79B-A8303E76B211}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7290" yWindow="-21285" windowWidth="30255" windowHeight="16650" xr2:uid="{B3EEA080-4589-4824-92D0-D334717E2C8E}"/>
   </bookViews>
@@ -27,30 +27,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Today</t>
   </si>
@@ -197,6 +175,9 @@
   </si>
   <si>
     <t>Float w/ callability</t>
+  </si>
+  <si>
+    <t>{=qlScheduleDates(B18)}</t>
   </si>
 </sst>
 </file>
@@ -240,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -256,6 +237,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -611,7 +595,7 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" cm="1">
+      <c r="B2" s="1">
         <f t="array" ref="B2">_xll.qlSettingsSetEvaluationDate(B1)</f>
         <v>46174</v>
       </c>
@@ -638,7 +622,7 @@
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="str" cm="1">
+      <c r="B6" s="2" t="str">
         <f t="array" ref="B6">_xll.qlBlackConstantVol(B2,"NullCalendar",0.25,"Act/365")</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R6C2BlackVolTermStructureHandle,A</v>
       </c>
@@ -655,7 +639,7 @@
       <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="2" t="str" cm="1">
+      <c r="B9" s="2" t="str">
         <f t="array" ref="B9">_xll.qlGeneralizedBlackScholesProcess(B7,B5,B4,B6)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R9C2GeneralizedBlackScholesProcess,A</v>
       </c>
@@ -673,7 +657,7 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="2" t="str" cm="1">
+      <c r="B13" s="2" t="str">
         <f t="array" ref="B13">_xll.qlEuribor("3m",B12)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R13C2Euribor,A</v>
       </c>
@@ -682,7 +666,7 @@
       <c r="A16" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="1" cm="1">
+      <c r="B16" s="1">
         <f t="array" ref="B16">_xll.qlCalendarAdvance("NullCalendar",B2,"5y")</f>
         <v>48000</v>
       </c>
@@ -691,7 +675,7 @@
       <c r="A17" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="1" cm="1">
+      <c r="B17" s="1">
         <f t="array" ref="B17">_xll.qlCalendarAdvance("NullCalendar",B2,"9y")</f>
         <v>49461</v>
       </c>
@@ -700,42 +684,36 @@
       <c r="A18" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="1" t="str" cm="1">
+      <c r="B18" s="1" t="str">
         <f t="array" ref="B18">_xll.qlMakeSchedule(B16,B17,"1y",,"Target")</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R18C2Schedule,A</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="B19" s="1" cm="1">
-        <f t="array" ref="B19:B23">_xll.qlScheduleDates(B18)</f>
+      <c r="B19" s="1">
+        <f>_xll.qlScheduleDates(B18)</f>
         <v>48001</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="B20" s="1">
-        <v>48366</v>
+      <c r="B20" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="B21" s="1">
-        <v>48731</v>
-      </c>
+      <c r="B21" s="1"/>
     </row>
     <row r="22" spans="1:2">
-      <c r="B22" s="1">
-        <v>49096</v>
-      </c>
+      <c r="B22" s="1"/>
     </row>
     <row r="23" spans="1:2">
-      <c r="B23" s="1">
-        <v>49461</v>
-      </c>
+      <c r="B23" s="1"/>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="2" t="str" cm="1">
+      <c r="B24" s="2" t="str">
         <f t="array" ref="B24">_xll.qlBermudanExercise(B19:B23)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R24C2BermudanExercise,A</v>
       </c>
@@ -744,7 +722,7 @@
       <c r="A25" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="2" t="str" cm="1">
+      <c r="B25" s="2" t="str">
         <f t="array" ref="B25">_xll.qlEuropeanExercise(B16)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R25C2EuropeanExercise,A</v>
       </c>
@@ -761,13 +739,13 @@
       <c r="A27" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="2" t="str" cm="1">
+      <c r="B27" s="2" t="str">
         <f t="array" ref="B27">_xll.qlCallability(_xll.qlBondPrice(100,"Clean"),"call",B19)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R27C2Callability,A</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="B28" s="2" t="str" cm="1">
+      <c r="B28" s="2" t="str">
         <f t="array" ref="B28">_xll.qlCallability(_xll.qlBondPrice(100,"Clean"),"call",B21)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R28C2Callability,A</v>
       </c>
@@ -801,7 +779,7 @@
       <c r="A32" t="s">
         <v>19</v>
       </c>
-      <c r="B32" s="1" cm="1">
+      <c r="B32" s="1">
         <f t="array" ref="B32">_xll.qlCalendarAdvance("Target",B29,"10y")</f>
         <v>49837</v>
       </c>
@@ -810,7 +788,7 @@
       <c r="A33" t="s">
         <v>20</v>
       </c>
-      <c r="B33" s="2" t="str" cm="1">
+      <c r="B33" s="2" t="str">
         <f t="array" ref="B33">_xll.qlMakeSchedule(B29,B32,"1y",,"Target")</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R33C2Schedule,A</v>
       </c>
@@ -819,7 +797,7 @@
       <c r="A34" t="s">
         <v>21</v>
       </c>
-      <c r="B34" s="2" t="str" cm="1">
+      <c r="B34" s="2" t="str">
         <f t="array" ref="B34">_xll.qlMakeSchedule(B29,B32,"3m",,"Target")</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R34C2Schedule,A</v>
       </c>
@@ -836,7 +814,7 @@
       <c r="A37" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="2" t="str" cm="1">
+      <c r="B37" s="2" t="str">
         <f t="array" ref="B37">_xll.qlConvertibleZeroCouponBond(B24,B26,B29,B30,"30/360",B33,B35)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R37C2ConvertibleZeroCouponBond,A</v>
       </c>
@@ -845,7 +823,7 @@
       <c r="A38" t="s">
         <v>23</v>
       </c>
-      <c r="B38" s="2" t="str" cm="1">
+      <c r="B38" s="2" t="str">
         <f t="array" ref="B38">_xll.qlConvertibleZeroCouponBond(B24,B26,B29,B30,"30/360",B33,B35,B27:B28)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R38C2ConvertibleZeroCouponBond,A</v>
       </c>
@@ -854,8 +832,8 @@
       <c r="A40" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="str" cm="1">
-        <f t="array" ref="B40">_xll.qlConvertibleFixedCouponBond(B24,B26,B29,B30,0.03,"30/360",B33,B35)</f>
+      <c r="B40" s="2" t="str">
+        <f t="array" ref="B40">_xll.qlConvertibleFixedCouponBond(B24,B26,B29,B30,0.03,"30/360",B33,B35,"0D","Target")</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R40C2ConvertibleFixedCouponBond,A</v>
       </c>
     </row>
@@ -863,8 +841,8 @@
       <c r="A41" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="str" cm="1">
-        <f t="array" ref="B41">_xll.qlConvertibleFixedCouponBond(B24,B26,B29,B30,0.03,"30/360",B33,B35,,,,,B27:B28)</f>
+      <c r="B41" s="2" t="str">
+        <f t="array" ref="B41">_xll.qlConvertibleFixedCouponBond(B24,B26,B29,B30,0.03,"30/360",B33,B35,"0D","Target",,,B27:B28)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R41C2ConvertibleFixedCouponBond,A</v>
       </c>
     </row>
@@ -872,8 +850,8 @@
       <c r="A43" t="s">
         <v>45</v>
       </c>
-      <c r="B43" s="2" t="str" cm="1">
-        <f t="array" ref="B43">_xll.qlConvertibleFloatingRateBond(B24,B26,B29,B30,B13,B31,0,"Act/360",B34,B35)</f>
+      <c r="B43" s="2" t="str">
+        <f t="array" ref="B43">_xll.qlConvertibleFloatingRateBond(B24,B26,B29,B30,B13,B31,0,"Act/360",B34,B35,"0D","Target")</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R43C2ConvertibleFloatingRateBond,A</v>
       </c>
     </row>
@@ -881,8 +859,8 @@
       <c r="A44" t="s">
         <v>46</v>
       </c>
-      <c r="B44" s="2" t="str" cm="1">
-        <f t="array" ref="B44">_xll.qlConvertibleFloatingRateBond(B24,B26,B29,B30,B13,B31,0,"Act/360",B34,B35,,,,,B27:B28)</f>
+      <c r="B44" s="2" t="str">
+        <f t="array" ref="B44">_xll.qlConvertibleFloatingRateBond(B24,B26,B29,B30,B13,B31,0,"Act/360",B34,B35,"0D","Target",,,B27:B28)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R44C2ConvertibleFloatingRateBond,A</v>
       </c>
     </row>
@@ -948,7 +926,7 @@
       <c r="A52" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B52" s="2" t="str" cm="1">
+      <c r="B52" s="2" t="str">
         <f t="array" ref="B52">_xll.qlBinomialConvertibleEngine(B47,B48,B49,B50)</f>
         <v>欣[test_convertiblebonds.xlsx]Sheet1!R52C2BinomialCRRConvertibleEngine,A</v>
       </c>
@@ -962,54 +940,54 @@
       <c r="A55" t="s">
         <v>41</v>
       </c>
-      <c r="B55" s="6" cm="1">
+      <c r="B55" s="6">
         <f t="array" ref="B55">_xll.qlInstrumentNPV(B37,_xll.qlInstrumentSetPricingEngine(B37,$B$52))</f>
-        <v>11046.869977387039</v>
+        <v>11081.337113450401</v>
       </c>
     </row>
     <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>42</v>
       </c>
-      <c r="B56" s="6" cm="1">
+      <c r="B56" s="6">
         <f t="array" ref="B56">_xll.qlInstrumentNPV(B38,_xll.qlInstrumentSetPricingEngine(B38,$B$52))</f>
-        <v>9519.443481791357</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>43</v>
       </c>
-      <c r="B57" s="6" cm="1">
+      <c r="B57" s="6">
         <f t="array" ref="B57">_xll.qlInstrumentNPV(B40,_xll.qlInstrumentSetPricingEngine(B40,$B$52))</f>
-        <v>11067.80952084887</v>
+        <v>11101.465444821617</v>
       </c>
     </row>
     <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>44</v>
       </c>
-      <c r="B58" s="6" cm="1">
+      <c r="B58" s="6">
         <f t="array" ref="B58">_xll.qlInstrumentNPV(B41,_xll.qlInstrumentSetPricingEngine(B41,$B$52))</f>
-        <v>9530.587049288697</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="59" spans="1:7">
       <c r="A59" t="s">
         <v>47</v>
       </c>
-      <c r="B59" s="6" cm="1">
+      <c r="B59" s="6">
         <f t="array" ref="B59">_xll.qlInstrumentNPV(B43,_xll.qlInstrumentSetPricingEngine(B43,$B$52))</f>
-        <v>11068.96500408951</v>
+        <v>11102.529015531909</v>
       </c>
     </row>
     <row r="60" spans="1:7">
       <c r="A60" t="s">
         <v>48</v>
       </c>
-      <c r="B60" s="6" cm="1">
+      <c r="B60" s="6">
         <f t="array" ref="B60">_xll.qlInstrumentNPV(B44,_xll.qlInstrumentSetPricingEngine(B44,$B$52))</f>
-        <v>9532.7273553674495</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>